<commit_message>
Housekeeping: regenerated dialogue workbooks post-apply, settings cleanup
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/セリフ編集/_キャラ対応表.xlsx
+++ b/セリフ編集/_キャラ対応表.xlsx
@@ -272,17 +272,17 @@
       </c>
       <c r="F2" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="G2" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
     </row>
@@ -294,37 +294,37 @@
       </c>
       <c r="B3" t="inlineStr" s="13">
         <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="13">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="13">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="13">
+        <is>
           <t xml:space="preserve">8</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="13">
+      <c r="F3" t="inlineStr" s="12">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="13">
         <is>
           <t xml:space="preserve">3</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr" s="13">
+      <c r="H3" t="inlineStr" s="13">
         <is>
           <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr" s="13">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr" s="12">
-        <is>
-          <t xml:space="preserve">0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr" s="13">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr" s="13">
-        <is>
-          <t xml:space="preserve">2</t>
         </is>
       </c>
     </row>
@@ -408,7 +408,7 @@
       </c>
       <c r="H5" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
     </row>
@@ -445,7 +445,7 @@
       </c>
       <c r="G6" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="H6" t="inlineStr" s="13">
@@ -487,12 +487,12 @@
       </c>
       <c r="G7" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">12</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="D2" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">深町真琴、相沢未来、小森さなえ、浜竹美咲、椿山みさき、三浦早紀</t>
+          <t xml:space="preserve">深町真琴、相沢未来、浜竹美咲、椿山みさき、南谷杏、三浦早紀</t>
         </is>
       </c>
     </row>
@@ -612,12 +612,12 @@
       </c>
       <c r="C3" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">高津小春、園部梨花、上野原弥生、丹羽穂垂、大庭愛菜、南谷杏、赤羽あんな、木村レイカ</t>
+          <t xml:space="preserve">高津小春、園部梨花、上野原弥生、丹羽穂垂、大庭愛菜、赤羽あんな、木村レイカ</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="D6" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">宇田川里奈、松川杏樹、早川モナ、海老名栞、坂本莉衣奈、リナ・モーガン</t>
+          <t xml:space="preserve">宇田川里奈、松川杏樹、小森さなえ、早川モナ、坂本莉衣奈、リナ・モーガン</t>
         </is>
       </c>
     </row>
@@ -766,12 +766,12 @@
       </c>
       <c r="C10" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">斎藤麻衣、菊池璃子、須藤美月</t>
+          <t xml:space="preserve">斎藤麻衣、菊池璃子、須藤美月、山本理香</t>
         </is>
       </c>
     </row>
@@ -1206,12 +1206,12 @@
       </c>
       <c r="C30" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">西川ちあき、赤沼紗稀、松岡綾乃、柳沼英子</t>
+          <t xml:space="preserve">西川ちあき、赤沼紗稀、柳沼英子</t>
         </is>
       </c>
     </row>
@@ -1360,12 +1360,12 @@
       </c>
       <c r="C37" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">橘玲美、片桐ありさ、長谷川レオナ、山本理香</t>
+          <t xml:space="preserve">橘玲美、片桐ありさ</t>
         </is>
       </c>
     </row>
@@ -1448,12 +1448,12 @@
       </c>
       <c r="C41" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">根岸亞里亞、相田萌、三橋ふみえ、倉見菜々、愛川明日香</t>
+          <t xml:space="preserve">根岸亞里亞、相田萌、三橋ふみえ、倉見菜々、穴澤ほのか、海老名栞、愛川明日香</t>
         </is>
       </c>
     </row>
@@ -1470,12 +1470,12 @@
       </c>
       <c r="C42" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">新見ゆり、飯島冴子、小西ゆきえ</t>
+          <t xml:space="preserve">長谷川レオナ、新見ゆり、飯島冴子、小西ゆきえ</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="C44" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">澤出みずき、平松かなみ、柳島みずほ、穴澤ほのか、玉手すみれ、松久保伊織、米山杏里、土岐山乃ノ佳、結城玲奈</t>
+          <t xml:space="preserve">澤出みずき、平松かなみ、柳島みずほ、玉手すみれ、松久保伊織、米山杏里、土岐山乃ノ佳、結城玲奈</t>
         </is>
       </c>
     </row>
@@ -1536,12 +1536,12 @@
       </c>
       <c r="C45" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">白銀麗子、大久保桃子</t>
+          <t xml:space="preserve">大久保桃子</t>
         </is>
       </c>
     </row>
@@ -1580,12 +1580,12 @@
       </c>
       <c r="C47" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">黒江舞、阿部みのり、高島さや</t>
+          <t xml:space="preserve">黒江舞、阿部みのり、高島さや、松岡綾乃</t>
         </is>
       </c>
     </row>
@@ -1624,12 +1624,12 @@
       </c>
       <c r="C49" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">12</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="12">
         <is>
-          <t xml:space="preserve">高階まさみ、川野辺菜穂子、四条あずさ、宮守なつめ、高橋まゆみ、伊勢原文奈、富士見ヶ丘遥、栗林あかり、財津琴美、豊田いすず、榊原菜摘</t>
+          <t xml:space="preserve">高階まさみ、川野辺菜穂子、四条あずさ、宮守なつめ、白銀麗子、高橋まゆみ、伊勢原文奈、富士見ヶ丘遥、栗林あかり、財津琴美、豊田いすず、榊原菜摘</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="D37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">強気</t>
+          <t xml:space="preserve">真面目</t>
         </is>
       </c>
       <c r="E37" t="inlineStr" s="2">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="D53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ノーマル</t>
+          <t xml:space="preserve">お気楽</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="2">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="D66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ノーマル</t>
+          <t xml:space="preserve">真面目</t>
         </is>
       </c>
       <c r="E66" t="inlineStr" s="2">
@@ -4291,12 +4291,12 @@
       </c>
       <c r="C72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">丁寧</t>
+          <t xml:space="preserve">蠱惑</t>
         </is>
       </c>
       <c r="D72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ノーマル</t>
+          <t xml:space="preserve">お気楽</t>
         </is>
       </c>
       <c r="E72" t="inlineStr" s="2">
@@ -4402,7 +4402,7 @@
       </c>
       <c r="C75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">標準</t>
+          <t xml:space="preserve">蠱惑</t>
         </is>
       </c>
       <c r="D75" t="inlineStr" s="2">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="D84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">強気</t>
+          <t xml:space="preserve">ノーマル</t>
         </is>
       </c>
       <c r="E84" t="inlineStr" s="2">
@@ -5566,12 +5566,12 @@
       </c>
       <c r="C107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">クール</t>
+          <t xml:space="preserve">丁寧</t>
         </is>
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ノーマル</t>
+          <t xml:space="preserve">内気</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
@@ -6084,12 +6084,12 @@
       </c>
       <c r="C121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">蠱惑</t>
+          <t xml:space="preserve">鷹揚</t>
         </is>
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">ノーマル</t>
+          <t xml:space="preserve">強気</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">

</xml_diff>